<commit_message>
Update the code to suit .yaml with unique name
</commit_message>
<xml_diff>
--- a/reports/tables/model_summary_validation.xlsx
+++ b/reports/tables/model_summary_validation.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,17 +536,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Zero Return Baseline</t>
+          <t>4-Week Moving Average</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>zero</t>
+          <t>moving_average</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>zero_v1</t>
+          <t>ma_4w_v1</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -554,7 +554,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{'lookback_weeks': 4}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -571,57 +571,69 @@
         <v>520</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0327547949250214</v>
+        <v>0.0364741534488731</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0481335817864723</v>
-      </c>
-      <c r="K2" t="inlineStr"/>
+        <v>0.0519290804762313</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.5318725099601593</v>
+      </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>0.0084045395018139</v>
       </c>
       <c r="M2" t="n">
         <v>0.0074661154670936</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.0074661154670936</v>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+        <v>0.0009384240347203</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.07456865807613533</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.5384615384615384</v>
+      </c>
       <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.01221213479694135</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.007466115467093643</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.004746019329847721</v>
+      </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>outputs/backtests/zero_v1/2025-01-01_to_2025-12-31</t>
+          <t>outputs/backtests/ma_4w_v1/2025-01-01_to_2025-12-31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4-Week Moving Average</t>
+          <t>4-Week EWMA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>moving_average</t>
+          <t>ewma</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ma_4w_v1</t>
+          <t>ewma_span4_v1</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -629,7 +641,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{'lookback_weeks': 4}</t>
+          <t>{'span_weeks': 4}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -646,40 +658,40 @@
         <v>520</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0364741534488731</v>
+        <v>0.0367187623707043</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0519290804762313</v>
+        <v>0.0523255179674865</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5318725099601593</v>
+        <v>0.5179282868525896</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0084045395018139</v>
+        <v>0.0082878298377069</v>
       </c>
       <c r="M3" t="n">
         <v>0.0074661154670936</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0009384240347203</v>
+        <v>0.0008217143706132</v>
       </c>
       <c r="O3" t="n">
-        <v>0.07456865807613533</v>
+        <v>0.07994415526528267</v>
       </c>
       <c r="P3" t="n">
-        <v>0.5384615384615384</v>
+        <v>0.5</v>
       </c>
       <c r="Q3" t="n">
         <v>52</v>
       </c>
       <c r="R3" t="n">
-        <v>0.01221213479694135</v>
+        <v>0.01539884847319758</v>
       </c>
       <c r="S3" t="n">
         <v>0.007466115467093643</v>
       </c>
       <c r="T3" t="n">
-        <v>0.004746019329847721</v>
+        <v>0.007932733006103943</v>
       </c>
       <c r="U3" t="n">
         <v>52</v>
@@ -690,93 +702,6 @@
         </is>
       </c>
       <c r="W3" t="inlineStr">
-        <is>
-          <t>outputs/backtests/ma_4w_v1/2025-01-01_to_2025-12-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>4-Week EWMA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ewma</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ewma_span4_v1</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>{'span_weeks': 4}</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2025-01-01</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2025-12-31</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>520</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.0367187623707043</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.0523255179674865</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.5179282868525896</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.0082878298377069</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.0074661154670936</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.0008217143706132</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.07994415526528267</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>52</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.01539884847319758</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.007466115467093643</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.007932733006103943</v>
-      </c>
-      <c r="U4" t="n">
-        <v>52</v>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
         <is>
           <t>outputs/backtests/ewma_span4_v1/2025-01-01_to_2025-12-31</t>
         </is>

</xml_diff>

<commit_message>
add the ensemble ymal
</commit_message>
<xml_diff>
--- a/reports/tables/model_summary_validation.xlsx
+++ b/reports/tables/model_summary_validation.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3273,7 +3273,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Portfolio Router V1</t>
+          <t>Regression Optuna V1 Stable Portfolio</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3283,12 +3283,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>portfolio_router_v1</t>
+          <t>regression_optuna_v1_stable_portfolio</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1_stable</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3315,31 +3315,31 @@
         <v>350</v>
       </c>
       <c r="J44" t="n">
-        <v>0.0375191577486723</v>
+        <v>0.0358984212991958</v>
       </c>
       <c r="K44" t="n">
-        <v>0.0488894891130647</v>
+        <v>0.0470496345170988</v>
       </c>
       <c r="L44" t="n">
         <v>347</v>
       </c>
       <c r="M44" t="n">
-        <v>0.5360230547550432</v>
+        <v>0.5043227665706052</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0013603153747285</v>
+        <v>0.0042217627158701</v>
       </c>
       <c r="O44" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P44" t="n">
-        <v>-0.0009345650433709</v>
+        <v>0.0019268822977706</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Regression Optuna V1 Stable Portfolio</t>
+          <t>Regression Optuna V2 Stable Portfolio</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3349,12 +3349,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>regression_optuna_v1_stable_portfolio</t>
+          <t>regression_optuna_v2_stable_portfolio</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>v1_stable</t>
+          <t>v2_stable</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3381,56 +3381,56 @@
         <v>350</v>
       </c>
       <c r="J45" t="n">
-        <v>0.0358984212991958</v>
+        <v>0.0354757730668497</v>
       </c>
       <c r="K45" t="n">
-        <v>0.0470496345170988</v>
+        <v>0.0465193933055148</v>
       </c>
       <c r="L45" t="n">
         <v>347</v>
       </c>
       <c r="M45" t="n">
-        <v>0.5043227665706052</v>
+        <v>0.515850144092219</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0042217627158701</v>
+        <v>0.0031756429596331</v>
       </c>
       <c r="O45" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P45" t="n">
-        <v>0.0019268822977706</v>
+        <v>0.0008807625415336</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Regression Optuna V2 Stable Portfolio</t>
+          <t>Regression Global Portfolio Optuna V1 Best</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>portfolio_router</t>
+          <t>general_regression</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>regression_optuna_v2_stable_portfolio</t>
+          <t>regression_portfolio_mae_optuna_v1_best</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>v2_stable</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{'standardize': True, 'fit_intercept': True, 'max_iter': 30000, 'tol': 0.0001, 'estimator': 'lasso', 'minimum_training_weeks': 104, 'alpha': 0.006251373574521752}</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{'feature_set': 'weekly_v1', 'feature_map_path': 'data/processed/weekly_features_weekly_v1.csv', 'selected_columns': ['return_lag_1', 'return_lag_2', 'return_lag_3', 'return_lag_4', 'return_lag_8', 'return_lag_12', 'return_lag_24', 'return_lag_52', 'rolling_mean_4', 'rolling_std_4', 'downside_deviation_4', 'risk_adjusted_mean_4', 'rolling_mean_12', 'rolling_std_12', 'downside_deviation_12', 'risk_adjusted_mean_12', 'rolling_mean_26', 'rolling_std_26', 'downside_deviation_26', 'risk_adjusted_mean_26', 'momentum_spread_4_12', 'market_return_lag_1', 'market_rolling_mean_4', 'market_rolling_mean_12', 'market_rolling_mean_26', 'excess_return_lag_1', 'excess_return_lag_2', 'excess_return_lag_3', 'excess_return_lag_4', 'excess_return_lag_8', 'excess_return_lag_12', 'excess_return_lag_24', 'excess_return_lag_52', 'excess_rolling_mean_4', 'excess_rolling_mean_12', 'excess_rolling_mean_26', 'return_lag_1_cs_z', 'return_lag_4_cs_z', 'return_lag_12_cs_z', 'rolling_mean_4_cs_z', 'rolling_mean_12_cs_z', 'rolling_mean_26_cs_z', 'risk_adjusted_mean_4_cs_z', 'excess_return_lag_1_cs_z']}</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3447,31 +3447,31 @@
         <v>350</v>
       </c>
       <c r="J46" t="n">
-        <v>0.0354757730668497</v>
+        <v>0.035424644638625</v>
       </c>
       <c r="K46" t="n">
-        <v>0.0465193933055148</v>
+        <v>0.0465365365200903</v>
       </c>
       <c r="L46" t="n">
         <v>347</v>
       </c>
       <c r="M46" t="n">
-        <v>0.515850144092219</v>
+        <v>0.5273775216138329</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0031756429596331</v>
+        <v>0.0026301993208483</v>
       </c>
       <c r="O46" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P46" t="n">
-        <v>0.0008807625415336</v>
+        <v>0.0003353189027488</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Regression Global Portfolio Optuna V1 Best</t>
+          <t>Regression Global Portfolio Optuna V2 Best</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3481,12 +3481,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>regression_portfolio_mae_optuna_v1_best</t>
+          <t>regression_portfolio_mae_optuna_v2_best</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3537,32 +3537,32 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Regression Global Portfolio Optuna V2 Best</t>
+          <t>XGBoost Group V1 + Global V1 Ensemble</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>general_regression</t>
+          <t>ensemble</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>regression_portfolio_mae_optuna_v2_best</t>
+          <t>xgboost_group_global_v1_ensemble</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>group_global_v1</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>{'standardize': True, 'fit_intercept': True, 'max_iter': 30000, 'tol': 0.0001, 'estimator': 'lasso', 'minimum_training_weeks': 104, 'alpha': 0.006251373574521752}</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>{'feature_set': 'weekly_v1', 'feature_map_path': 'data/processed/weekly_features_weekly_v1.csv', 'selected_columns': ['return_lag_1', 'return_lag_2', 'return_lag_3', 'return_lag_4', 'return_lag_8', 'return_lag_12', 'return_lag_24', 'return_lag_52', 'rolling_mean_4', 'rolling_std_4', 'downside_deviation_4', 'risk_adjusted_mean_4', 'rolling_mean_12', 'rolling_std_12', 'downside_deviation_12', 'risk_adjusted_mean_12', 'rolling_mean_26', 'rolling_std_26', 'downside_deviation_26', 'risk_adjusted_mean_26', 'momentum_spread_4_12', 'market_return_lag_1', 'market_rolling_mean_4', 'market_rolling_mean_12', 'market_rolling_mean_26', 'excess_return_lag_1', 'excess_return_lag_2', 'excess_return_lag_3', 'excess_return_lag_4', 'excess_return_lag_8', 'excess_return_lag_12', 'excess_return_lag_24', 'excess_return_lag_52', 'excess_rolling_mean_4', 'excess_rolling_mean_12', 'excess_rolling_mean_26', 'return_lag_1_cs_z', 'return_lag_4_cs_z', 'return_lag_12_cs_z', 'rolling_mean_4_cs_z', 'rolling_mean_12_cs_z', 'rolling_mean_26_cs_z', 'risk_adjusted_mean_4_cs_z', 'excess_return_lag_1_cs_z']}</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3579,46 +3579,46 @@
         <v>350</v>
       </c>
       <c r="J48" t="n">
-        <v>0.035424644638625</v>
+        <v>0.0352649477635961</v>
       </c>
       <c r="K48" t="n">
-        <v>0.0465365365200903</v>
+        <v>0.0463093319136323</v>
       </c>
       <c r="L48" t="n">
         <v>347</v>
       </c>
       <c r="M48" t="n">
-        <v>0.5273775216138329</v>
+        <v>0.5389048991354467</v>
       </c>
       <c r="N48" t="n">
-        <v>0.0026301993208483</v>
+        <v>0.0028099658071602</v>
       </c>
       <c r="O48" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P48" t="n">
-        <v>0.0003353189027488</v>
+        <v>0.0005150853890607</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>XGBoost Optuna V1 Stable Portfolio</t>
+          <t>XGBoost Group V2 + Global V2 Ensemble</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>portfolio_router</t>
+          <t>ensemble</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>xgboost_optuna_v1_stable_portfolio</t>
+          <t>xgboost_group_global_v2_ensemble</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>v1_stable</t>
+          <t>group_global_v2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3645,31 +3645,31 @@
         <v>350</v>
       </c>
       <c r="J49" t="n">
-        <v>0.0352151368667415</v>
+        <v>0.0353315866165629</v>
       </c>
       <c r="K49" t="n">
-        <v>0.0461821491979327</v>
+        <v>0.0465454496745774</v>
       </c>
       <c r="L49" t="n">
         <v>347</v>
       </c>
       <c r="M49" t="n">
-        <v>0.5302593659942363</v>
+        <v>0.5273775216138329</v>
       </c>
       <c r="N49" t="n">
-        <v>0.0031387634154556</v>
+        <v>0.0030915854022974</v>
       </c>
       <c r="O49" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P49" t="n">
-        <v>0.0008438829973561</v>
+        <v>0.0007967049841979</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>XGBoost Optuna V2 Stable Portfolio</t>
+          <t>XGBoost Optuna V1 Stable Portfolio</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>xgboost_optuna_v2_stable_portfolio</t>
+          <t>xgboost_optuna_v1_stable_portfolio</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>v2_stable</t>
+          <t>v1_stable</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3711,56 +3711,56 @@
         <v>350</v>
       </c>
       <c r="J50" t="n">
-        <v>0.0354048219634062</v>
+        <v>0.0352151368667415</v>
       </c>
       <c r="K50" t="n">
-        <v>0.0466879697661682</v>
+        <v>0.0461821491979327</v>
       </c>
       <c r="L50" t="n">
         <v>347</v>
       </c>
       <c r="M50" t="n">
-        <v>0.5360230547550432</v>
+        <v>0.5302593659942363</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0036891972961841</v>
+        <v>0.0031387634154556</v>
       </c>
       <c r="O50" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P50" t="n">
-        <v>0.0013943168780846</v>
+        <v>0.0008438829973561</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>XGBoost Global Portfolio Optuna V1 Best</t>
+          <t>XGBoost Optuna V2 Stable Portfolio</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>tree_boosting</t>
+          <t>portfolio_router</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>xgboost_portfolio_mae_optuna_v1_best</t>
+          <t>xgboost_optuna_v2_stable_portfolio</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v2_stable</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>{'estimator': 'xgboost', 'random_state': 42, 'n_jobs': -1, 'n_estimators': 40, 'max_depth': 2, 'learning_rate': 0.006215742516004331, 'subsample': 0.6290363762692827, 'colsample_bytree': 0.7599508686050309, 'reg_alpha': 0.06765379173473812, 'reg_lambda': 0.03368479659829659, 'min_child_weight': 7, 'minimum_training_weeks': 104}</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>{'feature_set': 'weekly_v1', 'feature_map_path': 'data/processed/weekly_features_weekly_v1.csv', 'selected_columns': ['return_lag_1', 'return_lag_2', 'return_lag_3', 'return_lag_4', 'return_lag_8', 'return_lag_12', 'return_lag_24', 'return_lag_52', 'rolling_mean_4', 'rolling_std_4', 'downside_deviation_4', 'risk_adjusted_mean_4', 'rolling_mean_12', 'rolling_std_12', 'downside_deviation_12', 'risk_adjusted_mean_12', 'rolling_mean_26', 'rolling_std_26', 'downside_deviation_26', 'risk_adjusted_mean_26', 'momentum_spread_4_12', 'market_return_lag_1', 'market_rolling_mean_4', 'market_rolling_mean_12', 'market_rolling_mean_26', 'excess_return_lag_1', 'excess_return_lag_2', 'excess_return_lag_3', 'excess_return_lag_4', 'excess_return_lag_8', 'excess_return_lag_12', 'excess_return_lag_24', 'excess_return_lag_52', 'excess_rolling_mean_4', 'excess_rolling_mean_12', 'excess_rolling_mean_26', 'return_lag_1_cs_z', 'return_lag_4_cs_z', 'return_lag_12_cs_z', 'rolling_mean_4_cs_z', 'rolling_mean_12_cs_z', 'rolling_mean_26_cs_z', 'risk_adjusted_mean_4_cs_z', 'excess_return_lag_1_cs_z']}</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3777,31 +3777,31 @@
         <v>350</v>
       </c>
       <c r="J51" t="n">
-        <v>0.035402571344816</v>
+        <v>0.0354048219634062</v>
       </c>
       <c r="K51" t="n">
-        <v>0.0465039231647275</v>
+        <v>0.0466879697661682</v>
       </c>
       <c r="L51" t="n">
         <v>347</v>
       </c>
       <c r="M51" t="n">
-        <v>0.5273775216138329</v>
+        <v>0.5360230547550432</v>
       </c>
       <c r="N51" t="n">
-        <v>0.0024811681988649</v>
+        <v>0.0036891972961841</v>
       </c>
       <c r="O51" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P51" t="n">
-        <v>0.0001862877807653</v>
+        <v>0.0013943168780846</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>XGBoost Global Portfolio Optuna V2 Best</t>
+          <t>XGBoost Global Portfolio Optuna V1 Best</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3811,17 +3811,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>xgboost_portfolio_mae_optuna_v2_best</t>
+          <t>xgboost_portfolio_mae_optuna_v1_best</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>{'estimator': 'xgboost', 'random_state': 42, 'n_jobs': -1, 'n_estimators': 40, 'max_depth': 2, 'learning_rate': 0.0050810207611557, 'subsample': 0.65518407213237, 'colsample_bytree': 0.6904277810232377, 'reg_alpha': 0.005055584896629372, 'reg_lambda': 0.0978960123134593, 'min_child_weight': 3, 'minimum_training_weeks': 104}</t>
+          <t>{'estimator': 'xgboost', 'random_state': 42, 'n_jobs': -1, 'n_estimators': 40, 'max_depth': 2, 'learning_rate': 0.006215742516004331, 'subsample': 0.6290363762692827, 'colsample_bytree': 0.7599508686050309, 'reg_alpha': 0.06765379173473812, 'reg_lambda': 0.03368479659829659, 'min_child_weight': 7, 'minimum_training_weeks': 104}</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3843,10 +3843,10 @@
         <v>350</v>
       </c>
       <c r="J52" t="n">
-        <v>0.0354066704859173</v>
+        <v>0.035402571344816</v>
       </c>
       <c r="K52" t="n">
-        <v>0.0465085498664776</v>
+        <v>0.0465039231647275</v>
       </c>
       <c r="L52" t="n">
         <v>347</v>
@@ -3855,76 +3855,142 @@
         <v>0.5273775216138329</v>
       </c>
       <c r="N52" t="n">
-        <v>0.0024939735084106</v>
+        <v>0.0024811681988649</v>
       </c>
       <c r="O52" t="n">
         <v>0.0022948804180995</v>
       </c>
       <c r="P52" t="n">
-        <v>0.0001990930903111</v>
+        <v>0.0001862877807653</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>XGBoost Global Portfolio Optuna V2 Best</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>tree_boosting</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>xgboost_portfolio_mae_optuna_v2_best</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>{'estimator': 'xgboost', 'random_state': 42, 'n_jobs': -1, 'n_estimators': 40, 'max_depth': 2, 'learning_rate': 0.0050810207611557, 'subsample': 0.65518407213237, 'colsample_bytree': 0.6904277810232377, 'reg_alpha': 0.005055584896629372, 'reg_lambda': 0.0978960123134593, 'min_child_weight': 3, 'minimum_training_weeks': 104}</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>{'feature_set': 'weekly_v1', 'feature_map_path': 'data/processed/weekly_features_weekly_v1.csv', 'selected_columns': ['return_lag_1', 'return_lag_2', 'return_lag_3', 'return_lag_4', 'return_lag_8', 'return_lag_12', 'return_lag_24', 'return_lag_52', 'rolling_mean_4', 'rolling_std_4', 'downside_deviation_4', 'risk_adjusted_mean_4', 'rolling_mean_12', 'rolling_std_12', 'downside_deviation_12', 'risk_adjusted_mean_12', 'rolling_mean_26', 'rolling_std_26', 'downside_deviation_26', 'risk_adjusted_mean_26', 'momentum_spread_4_12', 'market_return_lag_1', 'market_rolling_mean_4', 'market_rolling_mean_12', 'market_rolling_mean_26', 'excess_return_lag_1', 'excess_return_lag_2', 'excess_return_lag_3', 'excess_return_lag_4', 'excess_return_lag_8', 'excess_return_lag_12', 'excess_return_lag_24', 'excess_return_lag_52', 'excess_rolling_mean_4', 'excess_rolling_mean_12', 'excess_rolling_mean_26', 'return_lag_1_cs_z', 'return_lag_4_cs_z', 'return_lag_12_cs_z', 'rolling_mean_4_cs_z', 'rolling_mean_12_cs_z', 'rolling_mean_26_cs_z', 'risk_adjusted_mean_4_cs_z', 'excess_return_lag_1_cs_z']}</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>350</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.0354066704859173</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.0465085498664776</v>
+      </c>
+      <c r="L53" t="n">
+        <v>347</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.5273775216138329</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0.0024939735084106</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.0022948804180995</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0.0001990930903111</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>Zero Return Baseline</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>zero</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>zero_v1</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I53" t="n">
-        <v>350</v>
-      </c>
-      <c r="J53" t="n">
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>350</v>
+      </c>
+      <c r="J54" t="n">
         <v>0.0354646915214358</v>
       </c>
-      <c r="K53" t="n">
+      <c r="K54" t="n">
         <v>0.0465682065772564</v>
       </c>
-      <c r="L53" t="n">
+      <c r="L54" t="n">
         <v>0</v>
       </c>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="n">
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="n">
         <v>0</v>
       </c>
-      <c r="O53" t="n">
-        <v>0.0022948804180995</v>
-      </c>
-      <c r="P53" t="n">
+      <c r="O54" t="n">
+        <v>0.0022948804180995</v>
+      </c>
+      <c r="P54" t="n">
         <v>-0.0022948804180995</v>
       </c>
     </row>

</xml_diff>